<commit_message>
Interesting trading strategy for Whitewater
</commit_message>
<xml_diff>
--- a/whitewater/data/master_aligned.xlsx
+++ b/whitewater/data/master_aligned.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/efh2/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/efh2/PyCharmProjects/QuantCode26/whitewater/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB9612BE-CF15-2146-B5F5-7D2C77679503}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{121F39C7-16D4-5348-85CD-C3835E151834}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="HH_daily" sheetId="1" r:id="rId1"/>
@@ -18,7 +18,20 @@
     <sheet name="demand" sheetId="3" r:id="rId3"/>
     <sheet name="inventory" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -36,9 +49,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -50,6 +63,15 @@
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -87,12 +109,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -21860,7 +21885,7 @@
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
     </row>
@@ -22141,7 +22166,7 @@
         <v>43435</v>
       </c>
       <c r="B36">
-        <v>95562</v>
+        <v>102426</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -22149,7 +22174,7 @@
         <v>43466</v>
       </c>
       <c r="B37">
-        <v>95748</v>
+        <v>106507</v>
       </c>
     </row>
     <row r="38" spans="1:2" x14ac:dyDescent="0.2">
@@ -22157,7 +22182,7 @@
         <v>43497</v>
       </c>
       <c r="B38">
-        <v>75564</v>
+        <v>79284</v>
       </c>
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.2">
@@ -22165,7 +22190,7 @@
         <v>43525</v>
       </c>
       <c r="B39">
-        <v>93602</v>
+        <v>113680</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.2">
@@ -22173,7 +22198,7 @@
         <v>43556</v>
       </c>
       <c r="B40">
-        <v>84065</v>
+        <v>103108</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.2">
@@ -22181,7 +22206,7 @@
         <v>43586</v>
       </c>
       <c r="B41">
-        <v>107005</v>
+        <v>124470</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -22189,7 +22214,7 @@
         <v>43617</v>
       </c>
       <c r="B42">
-        <v>97739</v>
+        <v>118781</v>
       </c>
     </row>
     <row r="43" spans="1:2" x14ac:dyDescent="0.2">
@@ -22197,7 +22222,7 @@
         <v>43647</v>
       </c>
       <c r="B43">
-        <v>95194</v>
+        <v>128880</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -22205,7 +22230,7 @@
         <v>43678</v>
       </c>
       <c r="B44">
-        <v>76669</v>
+        <v>107504</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -22213,7 +22238,7 @@
         <v>43709</v>
       </c>
       <c r="B45">
-        <v>95250</v>
+        <v>136377</v>
       </c>
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.2">
@@ -22221,7 +22246,7 @@
         <v>43739</v>
       </c>
       <c r="B46">
-        <v>107359</v>
+        <v>160040</v>
       </c>
     </row>
     <row r="47" spans="1:2" x14ac:dyDescent="0.2">
@@ -22229,7 +22254,7 @@
         <v>43770</v>
       </c>
       <c r="B47">
-        <v>106014</v>
+        <v>153080</v>
       </c>
     </row>
     <row r="48" spans="1:2" x14ac:dyDescent="0.2">
@@ -22237,7 +22262,7 @@
         <v>43800</v>
       </c>
       <c r="B48">
-        <v>108451</v>
+        <v>172467</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -22245,7 +22270,7 @@
         <v>43831</v>
       </c>
       <c r="B49">
-        <v>114283</v>
+        <v>196247</v>
       </c>
     </row>
     <row r="50" spans="1:2" x14ac:dyDescent="0.2">
@@ -22253,7 +22278,7 @@
         <v>43862</v>
       </c>
       <c r="B50">
-        <v>98008</v>
+        <v>177711</v>
       </c>
     </row>
     <row r="51" spans="1:2" x14ac:dyDescent="0.2">
@@ -22261,7 +22286,7 @@
         <v>43891</v>
       </c>
       <c r="B51">
-        <v>98021</v>
+        <v>186103</v>
       </c>
     </row>
     <row r="52" spans="1:2" x14ac:dyDescent="0.2">
@@ -22269,7 +22294,7 @@
         <v>43922</v>
       </c>
       <c r="B52">
-        <v>91733</v>
+        <v>157863</v>
       </c>
     </row>
     <row r="53" spans="1:2" x14ac:dyDescent="0.2">
@@ -22277,7 +22302,7 @@
         <v>43952</v>
       </c>
       <c r="B53">
-        <v>77635</v>
+        <v>129954</v>
       </c>
     </row>
     <row r="54" spans="1:2" x14ac:dyDescent="0.2">
@@ -22285,7 +22310,7 @@
         <v>43983</v>
       </c>
       <c r="B54">
-        <v>26910</v>
+        <v>50302</v>
       </c>
     </row>
     <row r="55" spans="1:2" x14ac:dyDescent="0.2">
@@ -22293,7 +22318,7 @@
         <v>44013</v>
       </c>
       <c r="B55">
-        <v>30230</v>
+        <v>44593</v>
       </c>
     </row>
     <row r="56" spans="1:2" x14ac:dyDescent="0.2">
@@ -22301,7 +22326,7 @@
         <v>44044</v>
       </c>
       <c r="B56">
-        <v>29316</v>
+        <v>57757</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.2">
@@ -22309,7 +22334,7 @@
         <v>44075</v>
       </c>
       <c r="B57">
-        <v>61674</v>
+        <v>130205</v>
       </c>
     </row>
     <row r="58" spans="1:2" x14ac:dyDescent="0.2">
@@ -22317,7 +22342,7 @@
         <v>44105</v>
       </c>
       <c r="B58">
-        <v>88331</v>
+        <v>186246</v>
       </c>
     </row>
     <row r="59" spans="1:2" x14ac:dyDescent="0.2">
@@ -22325,7 +22350,7 @@
         <v>44136</v>
       </c>
       <c r="B59">
-        <v>101396</v>
+        <v>200094</v>
       </c>
     </row>
     <row r="60" spans="1:2" x14ac:dyDescent="0.2">
@@ -22333,7 +22358,7 @@
         <v>44166</v>
       </c>
       <c r="B60">
-        <v>109365</v>
+        <v>219654</v>
       </c>
     </row>
     <row r="61" spans="1:2" x14ac:dyDescent="0.2">
@@ -22341,7 +22366,7 @@
         <v>44197</v>
       </c>
       <c r="B61">
-        <v>111069</v>
+        <v>229388</v>
       </c>
     </row>
     <row r="62" spans="1:2" x14ac:dyDescent="0.2">
@@ -22349,7 +22374,7 @@
         <v>44228</v>
       </c>
       <c r="B62">
-        <v>83808</v>
+        <v>147609</v>
       </c>
     </row>
     <row r="63" spans="1:2" x14ac:dyDescent="0.2">
@@ -22357,7 +22382,7 @@
         <v>44256</v>
       </c>
       <c r="B63">
-        <v>114128</v>
+        <v>240344</v>
       </c>
     </row>
     <row r="64" spans="1:2" x14ac:dyDescent="0.2">
@@ -22365,7 +22390,7 @@
         <v>44287</v>
       </c>
       <c r="B64">
-        <v>108858</v>
+        <v>229344</v>
       </c>
     </row>
     <row r="65" spans="1:2" x14ac:dyDescent="0.2">
@@ -22373,7 +22398,7 @@
         <v>44317</v>
       </c>
       <c r="B65">
-        <v>108224</v>
+        <v>230206</v>
       </c>
     </row>
     <row r="66" spans="1:2" x14ac:dyDescent="0.2">
@@ -22381,7 +22406,7 @@
         <v>44348</v>
       </c>
       <c r="B66">
-        <v>85813</v>
+        <v>205888</v>
       </c>
     </row>
     <row r="67" spans="1:2" x14ac:dyDescent="0.2">
@@ -22389,7 +22414,7 @@
         <v>44378</v>
       </c>
       <c r="B67">
-        <v>96748</v>
+        <v>218126</v>
       </c>
     </row>
     <row r="68" spans="1:2" x14ac:dyDescent="0.2">
@@ -22397,7 +22422,7 @@
         <v>44409</v>
       </c>
       <c r="B68">
-        <v>99325</v>
+        <v>226700</v>
       </c>
     </row>
     <row r="69" spans="1:2" x14ac:dyDescent="0.2">
@@ -22405,7 +22430,7 @@
         <v>44440</v>
       </c>
       <c r="B69">
-        <v>99615</v>
+        <v>212559</v>
       </c>
     </row>
     <row r="70" spans="1:2" x14ac:dyDescent="0.2">
@@ -22413,7 +22438,7 @@
         <v>44470</v>
       </c>
       <c r="B70">
-        <v>101288</v>
+        <v>226161</v>
       </c>
     </row>
     <row r="71" spans="1:2" x14ac:dyDescent="0.2">
@@ -22421,7 +22446,7 @@
         <v>44501</v>
       </c>
       <c r="B71">
-        <v>112754</v>
+        <v>220190</v>
       </c>
     </row>
     <row r="72" spans="1:2" x14ac:dyDescent="0.2">
@@ -22429,7 +22454,7 @@
         <v>44531</v>
       </c>
       <c r="B72">
-        <v>119053</v>
+        <v>250291</v>
       </c>
     </row>
     <row r="73" spans="1:2" x14ac:dyDescent="0.2">
@@ -22437,7 +22462,7 @@
         <v>44562</v>
       </c>
       <c r="B73">
-        <v>130131</v>
+        <v>260825</v>
       </c>
     </row>
     <row r="74" spans="1:2" x14ac:dyDescent="0.2">
@@ -22445,7 +22470,7 @@
         <v>44593</v>
       </c>
       <c r="B74">
-        <v>110916</v>
+        <v>231577</v>
       </c>
     </row>
     <row r="75" spans="1:2" x14ac:dyDescent="0.2">
@@ -22453,7 +22478,7 @@
         <v>44621</v>
       </c>
       <c r="B75">
-        <v>130486</v>
+        <v>255126</v>
       </c>
     </row>
     <row r="76" spans="1:2" x14ac:dyDescent="0.2">
@@ -22461,7 +22486,7 @@
         <v>44652</v>
       </c>
       <c r="B76">
-        <v>124560</v>
+        <v>222114</v>
       </c>
     </row>
     <row r="77" spans="1:2" x14ac:dyDescent="0.2">
@@ -22469,7 +22494,7 @@
         <v>44682</v>
       </c>
       <c r="B77">
-        <v>130733</v>
+        <v>256198</v>
       </c>
     </row>
     <row r="78" spans="1:2" x14ac:dyDescent="0.2">
@@ -22477,7 +22502,7 @@
         <v>44713</v>
       </c>
       <c r="B78">
-        <v>105690</v>
+        <v>186734</v>
       </c>
     </row>
     <row r="79" spans="1:2" x14ac:dyDescent="0.2">
@@ -22485,7 +22510,7 @@
         <v>44743</v>
       </c>
       <c r="B79">
-        <v>118542</v>
+        <v>181623</v>
       </c>
     </row>
     <row r="80" spans="1:2" x14ac:dyDescent="0.2">
@@ -22493,7 +22518,7 @@
         <v>44774</v>
       </c>
       <c r="B80">
-        <v>118672</v>
+        <v>182080</v>
       </c>
     </row>
     <row r="81" spans="1:2" x14ac:dyDescent="0.2">
@@ -22501,7 +22526,7 @@
         <v>44805</v>
       </c>
       <c r="B81">
-        <v>115637</v>
+        <v>175448</v>
       </c>
     </row>
     <row r="82" spans="1:2" x14ac:dyDescent="0.2">
@@ -22509,7 +22534,7 @@
         <v>44835</v>
       </c>
       <c r="B82">
-        <v>130421</v>
+        <v>197207</v>
       </c>
     </row>
     <row r="83" spans="1:2" x14ac:dyDescent="0.2">
@@ -22517,7 +22542,7 @@
         <v>44866</v>
       </c>
       <c r="B83">
-        <v>120073</v>
+        <v>177101</v>
       </c>
     </row>
     <row r="84" spans="1:2" x14ac:dyDescent="0.2">
@@ -22525,7 +22550,7 @@
         <v>44896</v>
       </c>
       <c r="B84">
-        <v>139166</v>
+        <v>203285</v>
       </c>
     </row>
     <row r="85" spans="1:2" x14ac:dyDescent="0.2">
@@ -22533,7 +22558,7 @@
         <v>44927</v>
       </c>
       <c r="B85">
-        <v>139242</v>
+        <v>201810</v>
       </c>
     </row>
     <row r="86" spans="1:2" x14ac:dyDescent="0.2">
@@ -22541,7 +22566,7 @@
         <v>44958</v>
       </c>
       <c r="B86">
-        <v>119455</v>
+        <v>195125</v>
       </c>
     </row>
     <row r="87" spans="1:2" x14ac:dyDescent="0.2">
@@ -22549,7 +22574,7 @@
         <v>44986</v>
       </c>
       <c r="B87">
-        <v>130970</v>
+        <v>227093</v>
       </c>
     </row>
     <row r="88" spans="1:2" x14ac:dyDescent="0.2">
@@ -22557,7 +22582,7 @@
         <v>45017</v>
       </c>
       <c r="B88">
-        <v>136989</v>
+        <v>255058</v>
       </c>
     </row>
     <row r="89" spans="1:2" x14ac:dyDescent="0.2">
@@ -22565,7 +22590,7 @@
         <v>45047</v>
       </c>
       <c r="B89">
-        <v>126154</v>
+        <v>252300</v>
       </c>
     </row>
     <row r="90" spans="1:2" x14ac:dyDescent="0.2">
@@ -22573,7 +22598,7 @@
         <v>45078</v>
       </c>
       <c r="B90">
-        <v>83744</v>
+        <v>209481</v>
       </c>
     </row>
     <row r="91" spans="1:2" x14ac:dyDescent="0.2">
@@ -22581,7 +22606,7 @@
         <v>45108</v>
       </c>
       <c r="B91">
-        <v>113328</v>
+        <v>231489</v>
       </c>
     </row>
     <row r="92" spans="1:2" x14ac:dyDescent="0.2">
@@ -22589,7 +22614,7 @@
         <v>45139</v>
       </c>
       <c r="B92">
-        <v>118486</v>
+        <v>242356</v>
       </c>
     </row>
     <row r="93" spans="1:2" x14ac:dyDescent="0.2">
@@ -22597,7 +22622,7 @@
         <v>45170</v>
       </c>
       <c r="B93">
-        <v>115400</v>
+        <v>228780</v>
       </c>
     </row>
     <row r="94" spans="1:2" x14ac:dyDescent="0.2">
@@ -22605,7 +22630,7 @@
         <v>45200</v>
       </c>
       <c r="B94">
-        <v>132427</v>
+        <v>259764</v>
       </c>
     </row>
     <row r="95" spans="1:2" x14ac:dyDescent="0.2">
@@ -22613,7 +22638,7 @@
         <v>45231</v>
       </c>
       <c r="B95">
-        <v>130427</v>
+        <v>254981</v>
       </c>
     </row>
     <row r="96" spans="1:2" x14ac:dyDescent="0.2">
@@ -22621,7 +22646,7 @@
         <v>45261</v>
       </c>
       <c r="B96">
-        <v>141519</v>
+        <v>276932</v>
       </c>
     </row>
     <row r="97" spans="1:2" x14ac:dyDescent="0.2">
@@ -22629,7 +22654,7 @@
         <v>45292</v>
       </c>
       <c r="B97">
-        <v>137771</v>
+        <v>251615</v>
       </c>
     </row>
     <row r="98" spans="1:2" x14ac:dyDescent="0.2">
@@ -22637,7 +22662,7 @@
         <v>45323</v>
       </c>
       <c r="B98">
-        <v>128285</v>
+        <v>225513</v>
       </c>
     </row>
     <row r="99" spans="1:2" x14ac:dyDescent="0.2">
@@ -22645,7 +22670,7 @@
         <v>45352</v>
       </c>
       <c r="B99">
-        <v>138259</v>
+        <v>225783</v>
       </c>
     </row>
     <row r="100" spans="1:2" x14ac:dyDescent="0.2">
@@ -22653,7 +22678,7 @@
         <v>45383</v>
       </c>
       <c r="B100">
-        <v>119718</v>
+        <v>180583</v>
       </c>
     </row>
     <row r="101" spans="1:2" x14ac:dyDescent="0.2">
@@ -22661,7 +22686,7 @@
         <v>45413</v>
       </c>
       <c r="B101">
-        <v>131501</v>
+        <v>248247</v>
       </c>
     </row>
     <row r="102" spans="1:2" x14ac:dyDescent="0.2">
@@ -22669,7 +22694,7 @@
         <v>45444</v>
       </c>
       <c r="B102">
-        <v>108544</v>
+        <v>238069</v>
       </c>
     </row>
     <row r="103" spans="1:2" x14ac:dyDescent="0.2">
@@ -22677,7 +22702,7 @@
         <v>45474</v>
       </c>
       <c r="B103">
-        <v>119812</v>
+        <v>201963</v>
       </c>
     </row>
     <row r="104" spans="1:2" x14ac:dyDescent="0.2">
@@ -22685,7 +22710,7 @@
         <v>45505</v>
       </c>
       <c r="B104">
-        <v>118420</v>
+        <v>244860</v>
       </c>
     </row>
     <row r="105" spans="1:2" x14ac:dyDescent="0.2">
@@ -22693,7 +22718,7 @@
         <v>45536</v>
       </c>
       <c r="B105">
-        <v>121139</v>
+        <v>248761</v>
       </c>
     </row>
     <row r="106" spans="1:2" x14ac:dyDescent="0.2">
@@ -22701,7 +22726,7 @@
         <v>45566</v>
       </c>
       <c r="B106">
-        <v>128921</v>
+        <v>264732</v>
       </c>
     </row>
     <row r="107" spans="1:2" x14ac:dyDescent="0.2">
@@ -22709,7 +22734,7 @@
         <v>45597</v>
       </c>
       <c r="B107">
-        <v>126862</v>
+        <v>247972</v>
       </c>
     </row>
     <row r="108" spans="1:2" x14ac:dyDescent="0.2">
@@ -22717,7 +22742,7 @@
         <v>45627</v>
       </c>
       <c r="B108">
-        <v>133012</v>
+        <v>268377</v>
       </c>
     </row>
     <row r="109" spans="1:2" x14ac:dyDescent="0.2">
@@ -22725,7 +22750,7 @@
         <v>45658</v>
       </c>
       <c r="B109">
-        <v>138008</v>
+        <v>256157</v>
       </c>
     </row>
     <row r="110" spans="1:2" x14ac:dyDescent="0.2">
@@ -22733,7 +22758,7 @@
         <v>45689</v>
       </c>
       <c r="B110">
-        <v>117492</v>
+        <v>245569</v>
       </c>
     </row>
     <row r="111" spans="1:2" x14ac:dyDescent="0.2">
@@ -22741,7 +22766,7 @@
         <v>45717</v>
       </c>
       <c r="B111">
-        <v>137017</v>
+        <v>268094</v>
       </c>
     </row>
     <row r="112" spans="1:2" x14ac:dyDescent="0.2">
@@ -22749,7 +22774,7 @@
         <v>45748</v>
       </c>
       <c r="B112">
-        <v>127445</v>
+        <v>259957</v>
       </c>
     </row>
     <row r="113" spans="1:2" x14ac:dyDescent="0.2">
@@ -22757,7 +22782,7 @@
         <v>45778</v>
       </c>
       <c r="B113">
-        <v>124842</v>
+        <v>252702</v>
       </c>
     </row>
     <row r="114" spans="1:2" x14ac:dyDescent="0.2">
@@ -22765,7 +22790,7 @@
         <v>45809</v>
       </c>
       <c r="B114">
-        <v>84825</v>
+        <v>214190</v>
       </c>
     </row>
     <row r="115" spans="1:2" x14ac:dyDescent="0.2">
@@ -22773,7 +22798,7 @@
         <v>45839</v>
       </c>
       <c r="B115">
-        <v>114769</v>
+        <v>242671</v>
       </c>
     </row>
     <row r="116" spans="1:2" x14ac:dyDescent="0.2">
@@ -22781,7 +22806,7 @@
         <v>45870</v>
       </c>
       <c r="B116">
-        <v>118174</v>
+        <v>245250</v>
       </c>
     </row>
     <row r="117" spans="1:2" x14ac:dyDescent="0.2">
@@ -22789,7 +22814,7 @@
         <v>45901</v>
       </c>
       <c r="B117">
-        <v>116188</v>
+        <v>246227</v>
       </c>
     </row>
     <row r="118" spans="1:2" x14ac:dyDescent="0.2">
@@ -22797,7 +22822,7 @@
         <v>45931</v>
       </c>
       <c r="B118">
-        <v>127669</v>
+        <v>273611</v>
       </c>
     </row>
     <row r="119" spans="1:2" x14ac:dyDescent="0.2">
@@ -22805,7 +22830,7 @@
         <v>45962</v>
       </c>
       <c r="B119">
-        <v>135587</v>
+        <v>284776</v>
       </c>
     </row>
   </sheetData>

</xml_diff>